<commit_message>
2 order coils analysis
</commit_message>
<xml_diff>
--- a/tests/ITER_2D_APEC_evol_coils/input_template.xlsx
+++ b/tests/ITER_2D_APEC_evol_coils/input_template.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlasmaArc\tests\ITER_2D_APEC_evol_coils\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F6D3AB-B446-424E-A016-6CCCCF08CA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="element_types" sheetId="1" r:id="rId1"/>
-    <sheet name="dof_couplings" sheetId="2" r:id="rId2"/>
-    <sheet name="cpcyc" sheetId="3" r:id="rId3"/>
-    <sheet name="materials" sheetId="4" r:id="rId4"/>
-    <sheet name="real_constants" sheetId="5" r:id="rId5"/>
-    <sheet name="solver_settings" sheetId="6" r:id="rId6"/>
-    <sheet name="time_parameters" sheetId="7" r:id="rId7"/>
-    <sheet name="elem" sheetId="8" r:id="rId8"/>
-    <sheet name="node" sheetId="9" r:id="rId9"/>
-    <sheet name="transient_analysis" sheetId="10" r:id="rId10"/>
+    <sheet r:id="rId1" sheetId="1" name="element_types"/>
+    <sheet r:id="rId2" sheetId="2" name="dof_couplings"/>
+    <sheet r:id="rId3" sheetId="3" name="cpcyc"/>
+    <sheet r:id="rId4" sheetId="4" name="materials"/>
+    <sheet r:id="rId5" sheetId="5" name="real_constants"/>
+    <sheet r:id="rId6" sheetId="6" name="solver_settings"/>
+    <sheet r:id="rId7" sheetId="7" name="time_parameters"/>
+    <sheet r:id="rId8" sheetId="8" name="elem"/>
+    <sheet r:id="rId9" sheetId="9" name="node"/>
+    <sheet r:id="rId10" sheetId="10" name="transient_analysis"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -373,7 +367,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
@@ -419,44 +413,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="11">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -467,10 +464,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -508,71 +505,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -600,7 +597,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -623,11 +620,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -636,13 +633,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -652,7 +649,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -661,7 +658,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -670,7 +667,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -678,10 +675,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -746,23 +743,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="14.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -781,18 +782,18 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>112</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
       </c>
       <c r="D2" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="1">
         <v>1</v>
@@ -804,18 +805,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>112</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
       </c>
       <c r="D3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="1">
         <v>1</v>
@@ -827,18 +828,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>112</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
       </c>
       <c r="D4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
@@ -850,18 +851,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>112</v>
       </c>
       <c r="C5" s="1">
         <v>8</v>
       </c>
       <c r="D5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="1">
         <v>1</v>
@@ -879,24 +880,24 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="22.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="19.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="21.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="21.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -906,175 +907,175 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>1E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="2">
         <v>0.5</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="2">
-        <v>2.0000000000000001E-4</v>
+        <v>0.0002</v>
       </c>
       <c r="C3" s="1">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F3" s="2">
         <v>0.5</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0003</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F4" s="2">
         <v>0.5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>0.0004</v>
       </c>
       <c r="C5" s="1">
         <v>4</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="2">
         <v>0.5</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="2">
-        <v>5.0000000000000001E-4</v>
+        <v>0.0005</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="2">
         <v>0.5</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>6.0000000000000001E-3</v>
+        <v>0.006</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="2">
         <v>0.5</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1084,214 +1085,214 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1">
         <v>5</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1">
         <v>5</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1">
         <v>6</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1">
         <v>6</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1">
         <v>11</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1">
         <v>11</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1">
         <v>12</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1">
         <v>12</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1">
         <v>13</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="1">
         <v>13</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1">
         <v>14</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1">
         <v>14</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="1">
         <v>15</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="1">
         <v>15</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="1">
         <v>16</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="1">
         <v>16</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1301,57 +1302,68 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="14.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="7.147857142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="2"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1359,219 +1371,230 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="13" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>21</v>
       </c>
-      <c r="B2" s="7">
-        <v>1</v>
-      </c>
-      <c r="C2" s="7">
-        <v>1</v>
-      </c>
-      <c r="D2" s="7">
-        <v>1</v>
-      </c>
-      <c r="E2" s="7">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7">
-        <v>0</v>
-      </c>
-      <c r="J2" s="7">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9">
+        <v>1</v>
+      </c>
+      <c r="D2" s="9">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9">
+        <v>0</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9">
+        <v>0</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9">
+        <v>0</v>
+      </c>
+      <c r="K2" s="9">
+        <v>0</v>
+      </c>
+      <c r="L2" s="9">
+        <v>0</v>
+      </c>
+      <c r="M2" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>23</v>
       </c>
-      <c r="B3" s="7">
-        <v>1</v>
-      </c>
-      <c r="C3" s="7">
-        <v>1</v>
-      </c>
-      <c r="D3" s="7">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7">
-        <v>0</v>
-      </c>
-      <c r="G3" s="7">
-        <v>0</v>
-      </c>
-      <c r="H3" s="7">
-        <v>0</v>
-      </c>
-      <c r="I3" s="7">
-        <v>0</v>
-      </c>
-      <c r="J3" s="7">
-        <v>0</v>
-      </c>
-      <c r="K3" s="7">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7">
-        <v>0</v>
-      </c>
-      <c r="M3" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="9">
+        <v>1</v>
+      </c>
+      <c r="C3" s="9">
+        <v>1</v>
+      </c>
+      <c r="D3" s="9">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9">
+        <v>0</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0</v>
+      </c>
+      <c r="I3" s="9">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9">
+        <v>0</v>
+      </c>
+      <c r="K3" s="9">
+        <v>0</v>
+      </c>
+      <c r="L3" s="9">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>24</v>
       </c>
-      <c r="B4" s="7">
-        <v>1</v>
-      </c>
-      <c r="C4" s="7">
-        <v>1</v>
-      </c>
-      <c r="D4" s="7">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="F4" s="7">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="G4" s="7">
-        <v>7.9999999999999996E-7</v>
-      </c>
-      <c r="H4" s="7">
-        <v>0</v>
-      </c>
-      <c r="I4" s="7">
-        <v>0</v>
-      </c>
-      <c r="J4" s="7">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7">
-        <v>0</v>
-      </c>
-      <c r="L4" s="7">
-        <v>0</v>
-      </c>
-      <c r="M4" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9">
+        <v>8e-7</v>
+      </c>
+      <c r="F4" s="9">
+        <v>8e-7</v>
+      </c>
+      <c r="G4" s="9">
+        <v>8e-7</v>
+      </c>
+      <c r="H4" s="9">
+        <v>0</v>
+      </c>
+      <c r="I4" s="9">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9">
+        <v>0</v>
+      </c>
+      <c r="K4" s="9">
+        <v>0</v>
+      </c>
+      <c r="L4" s="9">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1">
         <v>25</v>
       </c>
-      <c r="B5" s="7">
-        <v>1</v>
-      </c>
-      <c r="C5" s="7">
-        <v>1</v>
-      </c>
-      <c r="D5" s="7">
-        <v>1</v>
-      </c>
-      <c r="E5" s="7">
-        <v>1E-8</v>
-      </c>
-      <c r="F5" s="7">
-        <v>1E-8</v>
-      </c>
-      <c r="G5" s="7">
-        <v>1E-8</v>
-      </c>
-      <c r="H5" s="7">
-        <v>0</v>
-      </c>
-      <c r="I5" s="7">
-        <v>0</v>
-      </c>
-      <c r="J5" s="7">
-        <v>0</v>
-      </c>
-      <c r="K5" s="7">
-        <v>0</v>
-      </c>
-      <c r="L5" s="7">
-        <v>0</v>
-      </c>
-      <c r="M5" s="7">
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9">
+        <v>1</v>
+      </c>
+      <c r="D5" s="9">
+        <v>1</v>
+      </c>
+      <c r="E5" s="9">
+        <v>1e-8</v>
+      </c>
+      <c r="F5" s="9">
+        <v>1e-8</v>
+      </c>
+      <c r="G5" s="9">
+        <v>1e-8</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9">
+        <v>0</v>
+      </c>
+      <c r="M5" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1581,30 +1604,45 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:V15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="9" width="6.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="6.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="22" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="21.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="10" width="12.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1625,7 +1663,7 @@
       <c r="I1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="9" t="s">
         <v>65</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -1665,15 +1703,15 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="7">
-        <v>0.94375189999999998</v>
+      <c r="C2" s="9">
+        <v>0.9437519</v>
       </c>
       <c r="D2" s="1">
         <v>249</v>
@@ -1693,8 +1731,8 @@
       <c r="I2" s="1">
         <v>-1</v>
       </c>
-      <c r="J2" s="7">
-        <v>1.6279714399999999E-2</v>
+      <c r="J2" s="9">
+        <v>0.0162797144</v>
       </c>
       <c r="K2" s="1">
         <v>1</v>
@@ -1733,15 +1771,15 @@
         <v>5732500</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
-      <c r="C3" s="7">
-        <v>0.41453946000000003</v>
+      <c r="C3" s="9">
+        <v>0.41453946</v>
       </c>
       <c r="D3" s="1">
         <v>116</v>
@@ -1750,7 +1788,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="2">
-        <v>8.2899999999999991</v>
+        <v>8.29</v>
       </c>
       <c r="G3" s="1">
         <v>0</v>
@@ -1761,8 +1799,8 @@
       <c r="I3" s="1">
         <v>-1</v>
       </c>
-      <c r="J3" s="7">
-        <v>1.6884624550000001E-2</v>
+      <c r="J3" s="9">
+        <v>0.01688462455</v>
       </c>
       <c r="K3" s="1">
         <v>1</v>
@@ -1801,15 +1839,15 @@
         <v>-2883400</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" s="7">
-        <v>0.66413093999999995</v>
+      <c r="C4" s="9">
+        <v>0.66413094</v>
       </c>
       <c r="D4" s="1">
         <v>186</v>
@@ -1829,8 +1867,8 @@
       <c r="I4" s="1">
         <v>-1</v>
       </c>
-      <c r="J4" s="7">
-        <v>3.9267408439999998E-2</v>
+      <c r="J4" s="9">
+        <v>0.03926740844</v>
       </c>
       <c r="K4" s="1">
         <v>1</v>
@@ -1869,15 +1907,15 @@
         <v>-5808400</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="7">
-        <v>0.60871516000000003</v>
+      <c r="C5" s="9">
+        <v>0.60871516</v>
       </c>
       <c r="D5" s="1">
         <v>170</v>
@@ -1897,8 +1935,8 @@
       <c r="I5" s="1">
         <v>-1</v>
       </c>
-      <c r="J5" s="7">
-        <v>3.56938854E-2</v>
+      <c r="J5" s="9">
+        <v>0.0356938854</v>
       </c>
       <c r="K5" s="1">
         <v>1</v>
@@ -1937,14 +1975,14 @@
         <v>-4776200</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="9">
         <v>0.7749625</v>
       </c>
       <c r="D6" s="1">
@@ -1965,8 +2003,8 @@
       <c r="I6" s="1">
         <v>-1</v>
       </c>
-      <c r="J6" s="7">
-        <v>3.1981995120000002E-2</v>
+      <c r="J6" s="9">
+        <v>0.03198199512</v>
       </c>
       <c r="K6" s="1">
         <v>1</v>
@@ -2005,14 +2043,14 @@
         <v>-7813300</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="9">
         <v>1.7265925</v>
       </c>
       <c r="D7" s="1">
@@ -2033,8 +2071,8 @@
       <c r="I7" s="1">
         <v>-1</v>
       </c>
-      <c r="J7" s="7">
-        <v>3.318021032E-2</v>
+      <c r="J7" s="9">
+        <v>0.03318021032</v>
       </c>
       <c r="K7" s="1">
         <v>1</v>
@@ -2073,14 +2111,14 @@
         <v>16941000</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1">
         <v>10</v>
       </c>
       <c r="B8" s="1">
         <v>1</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="9">
         <v>28.6027095</v>
       </c>
       <c r="D8" s="1">
@@ -2101,7 +2139,7 @@
       <c r="I8" s="1">
         <v>0</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <v>0</v>
       </c>
       <c r="K8" s="1">
@@ -2141,15 +2179,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1">
         <v>11</v>
       </c>
       <c r="B9" s="1">
         <v>1</v>
       </c>
-      <c r="C9" s="7">
-        <v>1.5560799999999999</v>
+      <c r="C9" s="9">
+        <v>1.55608</v>
       </c>
       <c r="D9" s="1">
         <v>553</v>
@@ -2169,8 +2207,8 @@
       <c r="I9" s="1">
         <v>-1</v>
       </c>
-      <c r="J9" s="7">
-        <v>2.0942284639999999E-2</v>
+      <c r="J9" s="9">
+        <v>0.02094228464</v>
       </c>
       <c r="K9" s="1">
         <v>1</v>
@@ -2209,15 +2247,15 @@
         <v>-4820400</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1">
         <v>12</v>
       </c>
       <c r="B10" s="1">
         <v>1</v>
       </c>
-      <c r="C10" s="7">
-        <v>1.5560799999999999</v>
+      <c r="C10" s="9">
+        <v>1.55608</v>
       </c>
       <c r="D10" s="1">
         <v>553</v>
@@ -2237,8 +2275,8 @@
       <c r="I10" s="1">
         <v>-1</v>
       </c>
-      <c r="J10" s="7">
-        <v>2.0942284639999999E-2</v>
+      <c r="J10" s="9">
+        <v>0.02094228464</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
@@ -2277,15 +2315,15 @@
         <v>-4048000</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1">
         <v>13</v>
       </c>
       <c r="B11" s="1">
         <v>1</v>
       </c>
-      <c r="C11" s="7">
-        <v>1.5560799999999999</v>
+      <c r="C11" s="9">
+        <v>1.55608</v>
       </c>
       <c r="D11" s="1">
         <v>553</v>
@@ -2305,8 +2343,8 @@
       <c r="I11" s="1">
         <v>-1</v>
       </c>
-      <c r="J11" s="7">
-        <v>2.0942284639999999E-2</v>
+      <c r="J11" s="9">
+        <v>0.02094228464</v>
       </c>
       <c r="K11" s="1">
         <v>1</v>
@@ -2345,15 +2383,15 @@
         <v>-20804000</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1">
         <v>14</v>
       </c>
       <c r="B12" s="1">
         <v>1</v>
       </c>
-      <c r="C12" s="7">
-        <v>1.5560799999999999</v>
+      <c r="C12" s="9">
+        <v>1.55608</v>
       </c>
       <c r="D12" s="1">
         <v>553</v>
@@ -2373,8 +2411,8 @@
       <c r="I12" s="1">
         <v>-1</v>
       </c>
-      <c r="J12" s="7">
-        <v>2.0942284639999999E-2</v>
+      <c r="J12" s="9">
+        <v>0.02094228464</v>
       </c>
       <c r="K12" s="1">
         <v>1</v>
@@ -2413,15 +2451,15 @@
         <v>-20804000</v>
       </c>
     </row>
-    <row r="13" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1">
         <v>15</v>
       </c>
       <c r="B13" s="1">
         <v>1</v>
       </c>
-      <c r="C13" s="7">
-        <v>1.5560799999999999</v>
+      <c r="C13" s="9">
+        <v>1.55608</v>
       </c>
       <c r="D13" s="1">
         <v>553</v>
@@ -2441,8 +2479,8 @@
       <c r="I13" s="1">
         <v>-1</v>
       </c>
-      <c r="J13" s="7">
-        <v>2.0942284639999999E-2</v>
+      <c r="J13" s="9">
+        <v>0.02094228464</v>
       </c>
       <c r="K13" s="1">
         <v>1</v>
@@ -2481,15 +2519,15 @@
         <v>-10297000</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1">
         <v>16</v>
       </c>
       <c r="B14" s="1">
         <v>1</v>
       </c>
-      <c r="C14" s="7">
-        <v>1.5560799999999999</v>
+      <c r="C14" s="9">
+        <v>1.55608</v>
       </c>
       <c r="D14" s="1">
         <v>553</v>
@@ -2509,8 +2547,8 @@
       <c r="I14" s="1">
         <v>-1</v>
       </c>
-      <c r="J14" s="7">
-        <v>2.0942284639999999E-2</v>
+      <c r="J14" s="9">
+        <v>0.02094228464</v>
       </c>
       <c r="K14" s="1">
         <v>1</v>
@@ -2549,14 +2587,14 @@
         <v>5301200</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1">
         <v>20</v>
       </c>
       <c r="B15" s="1">
         <v>1</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="9">
         <v>0</v>
       </c>
       <c r="D15" s="1">
@@ -2577,7 +2615,7 @@
       <c r="I15" s="1">
         <v>0</v>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="9">
         <v>0</v>
       </c>
       <c r="K15" s="1">
@@ -2623,279 +2661,279 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="6" width="34.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="12.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B4" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B5" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="7">
-        <v>1E-10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B6" s="9">
+        <v>1e-10</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B9" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B12" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B14" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B15" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B16" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="3" t="s">
         <v>39</v>
       </c>
       <c r="B17" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B18" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B21" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="3" t="s">
         <v>44</v>
       </c>
       <c r="B22" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B23" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B24" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="3" t="s">
         <v>47</v>
       </c>
       <c r="B25" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B27" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B28" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B29" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B30" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="3" t="s">
         <v>53</v>
       </c>
       <c r="B31" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B32" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="7">
-        <v>9.9999999999999995E-7</v>
+      <c r="B33" s="9">
+        <v>0.000001</v>
       </c>
     </row>
   </sheetData>
@@ -2904,75 +2942,75 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="6" width="23.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="11.290714285714287" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1">
@@ -2985,70 +3023,78 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="15.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="6.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="7"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="7"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="7"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="7"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="7"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="7"/>
+      <c r="B7" s="3"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="7"/>
+      <c r="B8" s="3"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="7"/>
+      <c r="B9" s="3"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
@@ -3058,95 +3104,108 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="16.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="17.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+      <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1"/>
+      <c r="B8" s="3"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1"/>
+      <c r="B9" s="3"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1"/>
+      <c r="B10" s="3"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1"/>
+      <c r="B12" s="3"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1"/>
+      <c r="B13" s="3"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>

</xml_diff>